<commit_message>
Update draw-tape specs in Excel/CSV/JSON and draw-tape.html to match official 台塑拉繩清潔袋 packaging specs
</commit_message>
<xml_diff>
--- a/src/data/inteplast_products_database.xlsx
+++ b/src/data/inteplast_products_database.xlsx
@@ -828,16 +828,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1186,27 +1186,27 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>13 Gallon</t>
+          <t>45L 大</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>60.9 × 68.5 cm</t>
+          <t>65 × 75 cm</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>經濟包</t>
+          <t>24張 / 經濟包</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>白色+拉繩</t>
+          <t>黑 / 透明</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>一拉即束打包/美式標準</t>
+          <t>台塑拉繩清潔袋 / 雙向抽拉打包</t>
         </is>
       </c>
     </row>
@@ -1223,27 +1223,27 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>30 Gallon</t>
+          <t>70L 特大</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>76.2 × 91.4 cm</t>
+          <t>78 × 88 cm</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>超量包</t>
+          <t>18張 / 經濟包</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>白色+拉繩</t>
+          <t>黑 / 透明</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>商業機構/大容量打包</t>
+          <t>台塑拉繩清潔袋 / 雙向抽拉打包</t>
         </is>
       </c>
     </row>
@@ -1260,508 +1260,508 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>醫療黃/紅色隔離袋</t>
+          <t>90L 超大</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>依需求客製</t>
+          <t>84 × 95 cm</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>警示印製</t>
+          <t>14張 / 經濟包</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>黃色 / 紅色</t>
+          <t>黑 / 透明</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>醫療傳染廢棄物隔離專用</t>
+          <t>台塑拉繩清潔袋 / 雙向抽拉打包</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>耐熱袋系列</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>四兩</t>
+          <t>90L 超大 (超量包)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>12.7 × 17.8 cm</t>
+          <t>84 × 95 cm</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>平裝 / 捲裝</t>
+          <t>25張 / 超量包</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>透明食品級</t>
+          <t>黑 / 透明</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>醬料/小份量食材打包</t>
+          <t>台塑拉繩清潔袋 / 雙向抽拉打包</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>耐熱袋系列</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>半斤</t>
+          <t>125L 超特大</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>15.2 × 22.8 cm</t>
+          <t>93 × 100 cm</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>平裝 / 捲裝</t>
+          <t>15張 / 經濟包</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>透明食品級</t>
+          <t>黑 / 透明</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>小吃/醬料/生鮮分裝</t>
+          <t>台塑拉繩清潔袋 / 雙向抽拉打包</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>耐熱袋系列</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>1斤</t>
+          <t>130L 巨無霸</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>20.3 × 27.9 cm</t>
+          <t>94 × 102 cm</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>平裝 / 捲裝</t>
+          <t>20張 / 超量包</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>透明食品級</t>
+          <t>黑 / 透明</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>餐飲熱食打包</t>
+          <t>台塑拉繩清潔袋 / 雙向抽拉打包</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>耐熱袋系列</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2斤</t>
+          <t>90L 超大 (彩色版)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>25.4 × 35.5 cm</t>
+          <t>84 × 95 cm</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>平裝 / 捲裝</t>
+          <t>25張 / 超量包</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>透明食品級</t>
+          <t>藍 / 粉</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>外帶熱湯/生鮮肉品</t>
+          <t>台塑拉繩清潔袋 / 馬卡龍雙色</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>耐熱袋系列</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>3斤</t>
+          <t>90L 超大 (盒裝)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>30.4 × 43.1 cm</t>
+          <t>84 × 95 cm</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>平裝 / 捲裝</t>
+          <t>80張 / 盒裝</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>透明食品級</t>
+          <t>黑</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>大份量熱食打包</t>
+          <t>台塑拉繩清潔袋 / 抽取盒裝</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>耐熱袋系列</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>5斤</t>
+          <t>125L 超特大 (盒裝)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>35.5 × 50.8 cm</t>
+          <t>93 × 100 cm</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>平裝 / 捲裝</t>
+          <t>66張 / 盒裝</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>透明食品級</t>
+          <t>黑</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>商業備料/高溫高壓打包</t>
+          <t>台塑拉繩清潔袋 / 抽取盒裝</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>1號夾鏈袋</t>
+          <t>醫療黃/紅色隔離袋</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>5.0 × 7.0 cm</t>
+          <t>依需求客製</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>警示印製</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>黃色 / 紅色</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>小型飾品/藥品分裝</t>
+          <t>醫療廢棄物隔離專用</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>耐熱袋系列</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2號夾鏈袋</t>
+          <t>四兩</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>6.0 × 8.5 cm</t>
+          <t>12.7 × 17.8 cm</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>平裝 / 捲裝</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>透明食品級</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>零件/隨身藥包</t>
+          <t>醬料/小份量食材打包</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>耐熱袋系列</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>3號夾鏈袋</t>
+          <t>半斤</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>7.0 × 10.0 cm</t>
+          <t>15.2 × 22.8 cm</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>平裝 / 捲裝</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>透明食品級</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>卡片/小物收納</t>
+          <t>小吃/醬料/生鮮分裝</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>耐熱袋系列</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>4號夾鏈袋</t>
+          <t>1斤</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>8.5 × 12.0 cm</t>
+          <t>20.3 × 27.9 cm</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>平裝 / 捲裝</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>透明食品級</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>試用品/小文具</t>
+          <t>餐飲熱食打包</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>耐熱袋系列</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>5號夾鏈袋</t>
+          <t>2斤</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>10.0 × 14.0 cm</t>
+          <t>25.4 × 35.5 cm</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>平裝 / 捲裝</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>透明食品級</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>食材分裝/小點心</t>
+          <t>外帶熱湯/生鮮肉品</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>耐熱袋系列</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>6號夾鏈袋</t>
+          <t>3斤</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>12.0 × 17.0 cm</t>
+          <t>30.4 × 43.1 cm</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>平裝 / 捲裝</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>透明食品級</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>中型食材/口罩收納</t>
+          <t>大份量熱食打包</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>耐熱袋系列</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>7號夾鏈袋</t>
+          <t>5斤</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>14.0 × 20.0 cm</t>
+          <t>35.5 × 50.8 cm</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>平裝 / 捲裝</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>透明食品級</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>蔬果/冷凍食品</t>
+          <t>商業備料/高溫高壓打包</t>
         </is>
       </c>
     </row>
@@ -1778,12 +1778,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>8號夾鏈袋</t>
+          <t>1號夾鏈袋</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>17.0 × 24.0 cm</t>
+          <t>5.0 × 7.0 cm</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>A5文件/冷凍肉品</t>
+          <t>小型飾品/藥品分裝</t>
         </is>
       </c>
     </row>
@@ -1815,12 +1815,12 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>9號夾鏈袋</t>
+          <t>2號夾鏈袋</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>20.0 × 28.0 cm</t>
+          <t>6.0 × 8.5 cm</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>服飾/大份量食材</t>
+          <t>零件/隨身藥包</t>
         </is>
       </c>
     </row>
@@ -1852,12 +1852,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>10號夾鏈袋</t>
+          <t>3號夾鏈袋</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>24.0 × 34.0 cm</t>
+          <t>7.0 × 10.0 cm</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>A4文件/大物件</t>
+          <t>卡片/小物收納</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>11號夾鏈袋</t>
+          <t>4號夾鏈袋</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>28.0 × 40.0 cm</t>
+          <t>8.5 × 12.0 cm</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>大件衣物/收納</t>
+          <t>試用品/小文具</t>
         </is>
       </c>
     </row>
@@ -1926,12 +1926,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>12號夾鏈袋</t>
+          <t>5號夾鏈袋</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>34.0 × 45.0 cm</t>
+          <t>10.0 × 14.0 cm</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1946,266 +1946,266 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>超大物件收納</t>
+          <t>食材分裝/小點心</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>手套 S</t>
+          <t>6號夾鏈袋</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>手掌寬 ~8 cm</t>
+          <t>12.0 × 17.0 cm</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>每盒100入</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>半透明</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>個人衛生/餐飲備料</t>
+          <t>中型食材/口罩收納</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>手套 M</t>
+          <t>7號夾鏈袋</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>手掌寬 ~9 cm</t>
+          <t>14.0 × 20.0 cm</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>每盒100入</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>半透明</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>個人衛生/餐飲備料</t>
+          <t>蔬果/冷凍食品</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>手套 L</t>
+          <t>8號夾鏈袋</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>手掌寬 ~10 cm</t>
+          <t>17.0 × 24.0 cm</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>每盒100入</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>半透明</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>個人衛生/餐飲備料</t>
+          <t>A5文件/冷凍肉品</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>手套 XL</t>
+          <t>9號夾鏈袋</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>手掌寬 ~11 cm</t>
+          <t>20.0 × 28.0 cm</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>每盒100入</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>半透明</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>個人衛生/餐飲備料</t>
+          <t>服飾/大份量食材</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>防塵膠帶 550mm</t>
+          <t>10號夾鏈袋</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>550 mm × 25 y (22.8m)</t>
+          <t>24.0 × 34.0 cm</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>卷裝</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>綠色膠帶+高密度膜</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>建築施工/小面積家具遮蔽</t>
+          <t>A4文件/大物件</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>防塵膠帶 1100mm</t>
+          <t>11號夾鏈袋</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>1100 mm × 25 y (22.8m)</t>
+          <t>28.0 × 40.0 cm</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>卷裝</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>綠色膠帶+高密度膜</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>裝潢養生/牆面家具遮蔽</t>
+          <t>大件衣物/收納</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>防塵膠帶 1500mm</t>
+          <t>12號夾鏈袋</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>1500 mm × 25 y (22.8m)</t>
+          <t>34.0 × 45.0 cm</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>卷裝</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>綠色膠帶+高密度膜</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>裝潢養生/牆面門窗遮蔽</t>
+          <t>超大物件收納</t>
         </is>
       </c>
     </row>
@@ -2222,27 +2222,27 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>防塵膠帶 2100mm</t>
+          <t>手套 S</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2100 mm × 25 y (22.8m)</t>
+          <t>手掌寬 ~8 cm</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>卷裝</t>
+          <t>每盒100入</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>綠色膠帶+高密度膜</t>
+          <t>半透明</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>門窗/大型家具大面積遮蔽</t>
+          <t>個人衛生/餐飲備料</t>
         </is>
       </c>
     </row>
@@ -2259,27 +2259,27 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>防塵膠帶 2700mm</t>
+          <t>手套 M</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>2700 mm × 25 y (22.8m)</t>
+          <t>手掌寬 ~9 cm</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>卷裝</t>
+          <t>每盒100入</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>綠色膠帶+高密度膜</t>
+          <t>半透明</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>工地工程/超大面積遮蔽</t>
+          <t>個人衛生/餐飲備料</t>
         </is>
       </c>
     </row>
@@ -2296,62 +2296,321 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>防塵膠帶 3200mm</t>
+          <t>手套 L</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>3200 mm × 25 y (22.8m)</t>
+          <t>手掌寬 ~10 cm</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>卷裝</t>
+          <t>每盒100入</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>綠色膠帶+高密度膜</t>
+          <t>半透明</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>工程施工/最大面積養生遮蔽</t>
+          <t>個人衛生/餐飲備料</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>手套 XL</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>手掌寬 ~11 cm</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>每盒100入</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>半透明</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>個人衛生/餐飲備料</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>防塵膠帶 550mm</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>550 mm × 25 y (22.8m)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>卷裝</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>綠色膠帶+高密度膜</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>建築施工/小面積家具遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>防塵膠帶 1100mm</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>1100 mm × 25 y (22.8m)</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>卷裝</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>綠色膠帶+高密度膜</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>裝潢養生/牆面家具遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>防塵膠帶 1500mm</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>1500 mm × 25 y (22.8m)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>卷裝</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>綠色膠帶+高密度膜</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>裝潢養生/牆面門窗遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>防塵膠帶 2100mm</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>2100 mm × 25 y (22.8m)</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>卷裝</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>綠色膠帶+高密度膜</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>門窗/大型家具大面積遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>防塵膠帶 2700mm</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>2700 mm × 25 y (22.8m)</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>卷裝</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>綠色膠帶+高密度膜</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>工地工程/超大面積遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>防塵膠帶 3200mm</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>3200 mm × 25 y (22.8m)</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>卷裝</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>綠色膠帶+高密度膜</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>工程施工/最大面積養生遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
           <t>006</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>Scale Sheet</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Scale Sheet</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>專案洽詢</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>專案對接</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>專案客製</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="G48" s="3" t="inlineStr">
         <is>
           <t>如有需求請聯繫專員專人對接</t>
         </is>

</xml_diff>

<commit_message>
Complete 5 medical drawtape bag sizes in Excel/CSV/JSON and restore exact red medical card styling
</commit_message>
<xml_diff>
--- a/src/data/inteplast_products_database.xlsx
+++ b/src/data/inteplast_products_database.xlsx
@@ -828,7 +828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -837,7 +837,7 @@
     <col width="27" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="33" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1519,175 +1519,175 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>醫療黃/紅色隔離袋</t>
+          <t>醫療袋 8L 小</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>依需求客製</t>
+          <t>39 × 40 cm</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>警示印製</t>
+          <t>40張 / 捲</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>黃色 / 紅色</t>
+          <t>紅</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>醫療廢棄物隔離專用</t>
+          <t>台塑拉繩醫療感染袋 / 感控隔離專用</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>耐熱袋系列</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>四兩</t>
+          <t>醫療袋 20L 中</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>12.7 × 17.8 cm</t>
+          <t>52 × 55 cm</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>平裝 / 捲裝</t>
+          <t>22張 / 捲</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>透明食品級</t>
+          <t>紅</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>醬料/小份量食材打包</t>
+          <t>台塑拉繩醫療感染袋 / 感控隔離專用</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>耐熱袋系列</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>半斤</t>
+          <t>醫療袋 50L 大</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>15.2 × 22.8 cm</t>
+          <t>69 × 78 cm</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>平裝 / 捲裝</t>
+          <t>12張 / 捲</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>透明食品級</t>
+          <t>紅</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>小吃/醬料/生鮮分裝</t>
+          <t>台塑拉繩醫療感染袋 / 感控隔離專用</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>耐熱袋系列</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>1斤</t>
+          <t>醫療袋 70L 特大</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>20.3 × 27.9 cm</t>
+          <t>77 × 92 cm</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>平裝 / 捲裝</t>
+          <t>8張 / 捲</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>透明食品級</t>
+          <t>紅</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>餐飲熱食打包</t>
+          <t>台塑拉繩醫療感染袋 / 感控隔離專用</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>耐熱袋系列</t>
+          <t>拉繩袋系列</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>2斤</t>
+          <t>醫療袋 90L 超大</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>25.4 × 35.5 cm</t>
+          <t>95 × 84 cm</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>平裝 / 捲裝</t>
+          <t>12張 / 捲</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>透明食品級</t>
+          <t>紅</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>外帶熱湯/生鮮肉品</t>
+          <t>台塑拉繩醫療感染袋 / 感控隔離專用</t>
         </is>
       </c>
     </row>
@@ -1704,12 +1704,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>3斤</t>
+          <t>四兩</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>30.4 × 43.1 cm</t>
+          <t>12.7 × 17.8 cm</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>大份量熱食打包</t>
+          <t>醬料/小份量食材打包</t>
         </is>
       </c>
     </row>
@@ -1741,12 +1741,12 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>5斤</t>
+          <t>半斤</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>35.5 × 50.8 cm</t>
+          <t>15.2 × 22.8 cm</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1761,155 +1761,155 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>商業備料/高溫高壓打包</t>
+          <t>小吃/醬料/生鮮分裝</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>耐熱袋系列</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>1號夾鏈袋</t>
+          <t>1斤</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>5.0 × 7.0 cm</t>
+          <t>20.3 × 27.9 cm</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>平裝 / 捲裝</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>透明食品級</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>小型飾品/藥品分裝</t>
+          <t>餐飲熱食打包</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>耐熱袋系列</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>2號夾鏈袋</t>
+          <t>2斤</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>6.0 × 8.5 cm</t>
+          <t>25.4 × 35.5 cm</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>平裝 / 捲裝</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>透明食品級</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>零件/隨身藥包</t>
+          <t>外帶熱湯/生鮮肉品</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>耐熱袋系列</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>3號夾鏈袋</t>
+          <t>3斤</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>7.0 × 10.0 cm</t>
+          <t>30.4 × 43.1 cm</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>平裝 / 捲裝</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>透明食品級</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>卡片/小物收納</t>
+          <t>大份量熱食打包</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>密封包裝類</t>
+          <t>耐熱袋系列</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>4號夾鏈袋</t>
+          <t>5斤</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>8.5 × 12.0 cm</t>
+          <t>35.5 × 50.8 cm</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>每包100入</t>
+          <t>平裝 / 捲裝</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>透明</t>
+          <t>透明食品級</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>試用品/小文具</t>
+          <t>商業備料/高溫高壓打包</t>
         </is>
       </c>
     </row>
@@ -1926,12 +1926,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>5號夾鏈袋</t>
+          <t>1號夾鏈袋</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>10.0 × 14.0 cm</t>
+          <t>5.0 × 7.0 cm</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>食材分裝/小點心</t>
+          <t>小型飾品/藥品分裝</t>
         </is>
       </c>
     </row>
@@ -1963,12 +1963,12 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>6號夾鏈袋</t>
+          <t>2號夾鏈袋</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>12.0 × 17.0 cm</t>
+          <t>6.0 × 8.5 cm</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>中型食材/口罩收納</t>
+          <t>零件/隨身藥包</t>
         </is>
       </c>
     </row>
@@ -2000,12 +2000,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>7號夾鏈袋</t>
+          <t>3號夾鏈袋</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>14.0 × 20.0 cm</t>
+          <t>7.0 × 10.0 cm</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>蔬果/冷凍食品</t>
+          <t>卡片/小物收納</t>
         </is>
       </c>
     </row>
@@ -2037,12 +2037,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>8號夾鏈袋</t>
+          <t>4號夾鏈袋</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>17.0 × 24.0 cm</t>
+          <t>8.5 × 12.0 cm</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>A5文件/冷凍肉品</t>
+          <t>試用品/小文具</t>
         </is>
       </c>
     </row>
@@ -2074,12 +2074,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>9號夾鏈袋</t>
+          <t>5號夾鏈袋</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>20.0 × 28.0 cm</t>
+          <t>10.0 × 14.0 cm</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>服飾/大份量食材</t>
+          <t>食材分裝/小點心</t>
         </is>
       </c>
     </row>
@@ -2111,12 +2111,12 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>10號夾鏈袋</t>
+          <t>6號夾鏈袋</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>24.0 × 34.0 cm</t>
+          <t>12.0 × 17.0 cm</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>A4文件/大物件</t>
+          <t>中型食材/口罩收納</t>
         </is>
       </c>
     </row>
@@ -2148,12 +2148,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>11號夾鏈袋</t>
+          <t>7號夾鏈袋</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>28.0 × 40.0 cm</t>
+          <t>14.0 × 20.0 cm</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>大件衣物/收納</t>
+          <t>蔬果/冷凍食品</t>
         </is>
       </c>
     </row>
@@ -2185,12 +2185,12 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>12號夾鏈袋</t>
+          <t>8號夾鏈袋</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>34.0 × 45.0 cm</t>
+          <t>17.0 × 24.0 cm</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -2205,155 +2205,155 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>超大物件收納</t>
+          <t>A5文件/冷凍肉品</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>手套 S</t>
+          <t>9號夾鏈袋</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>手掌寬 ~8 cm</t>
+          <t>20.0 × 28.0 cm</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>每盒100入</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>半透明</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>個人衛生/餐飲備料</t>
+          <t>服飾/大份量食材</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>手套 M</t>
+          <t>10號夾鏈袋</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>手掌寬 ~9 cm</t>
+          <t>24.0 × 34.0 cm</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>每盒100入</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>半透明</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>個人衛生/餐飲備料</t>
+          <t>A4文件/大物件</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>手套 L</t>
+          <t>11號夾鏈袋</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>手掌寬 ~10 cm</t>
+          <t>28.0 × 40.0 cm</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>每盒100入</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>半透明</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>個人衛生/餐飲備料</t>
+          <t>大件衣物/收納</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>其他類</t>
+          <t>密封包裝類</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>手套 XL</t>
+          <t>12號夾鏈袋</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>手掌寬 ~11 cm</t>
+          <t>34.0 × 45.0 cm</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>每盒100入</t>
+          <t>每包100入</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>半透明</t>
+          <t>透明</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>個人衛生/餐飲備料</t>
+          <t>超大物件收納</t>
         </is>
       </c>
     </row>
@@ -2370,27 +2370,27 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>防塵膠帶 550mm</t>
+          <t>手套 S</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>550 mm × 25 y (22.8m)</t>
+          <t>手掌寬 ~8 cm</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>卷裝</t>
+          <t>每盒100入</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>綠色膠帶+高密度膜</t>
+          <t>半透明</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>建築施工/小面積家具遮蔽</t>
+          <t>個人衛生/餐飲備料</t>
         </is>
       </c>
     </row>
@@ -2407,27 +2407,27 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>防塵膠帶 1100mm</t>
+          <t>手套 M</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>1100 mm × 25 y (22.8m)</t>
+          <t>手掌寬 ~9 cm</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>卷裝</t>
+          <t>每盒100入</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>綠色膠帶+高密度膜</t>
+          <t>半透明</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>裝潢養生/牆面家具遮蔽</t>
+          <t>個人衛生/餐飲備料</t>
         </is>
       </c>
     </row>
@@ -2444,27 +2444,27 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>防塵膠帶 1500mm</t>
+          <t>手套 L</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>1500 mm × 25 y (22.8m)</t>
+          <t>手掌寬 ~10 cm</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>卷裝</t>
+          <t>每盒100入</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>綠色膠帶+高密度膜</t>
+          <t>半透明</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>裝潢養生/牆面門窗遮蔽</t>
+          <t>個人衛生/餐飲備料</t>
         </is>
       </c>
     </row>
@@ -2481,27 +2481,27 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>防塵膠帶 2100mm</t>
+          <t>手套 XL</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>2100 mm × 25 y (22.8m)</t>
+          <t>手掌寬 ~11 cm</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>卷裝</t>
+          <t>每盒100入</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>綠色膠帶+高密度膜</t>
+          <t>半透明</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>門窗/大型家具大面積遮蔽</t>
+          <t>個人衛生/餐飲備料</t>
         </is>
       </c>
     </row>
@@ -2518,12 +2518,12 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>防塵膠帶 2700mm</t>
+          <t>防塵膠帶 550mm</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2700 mm × 25 y (22.8m)</t>
+          <t>550 mm × 25 y (22.8m)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>工地工程/超大面積遮蔽</t>
+          <t>建築施工/小面積家具遮蔽</t>
         </is>
       </c>
     </row>
@@ -2555,12 +2555,12 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>防塵膠帶 3200mm</t>
+          <t>防塵膠帶 1100mm</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>3200 mm × 25 y (22.8m)</t>
+          <t>1100 mm × 25 y (22.8m)</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -2575,42 +2575,190 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>工程施工/最大面積養生遮蔽</t>
+          <t>裝潢養生/牆面家具遮蔽</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>防塵膠帶 1500mm</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>1500 mm × 25 y (22.8m)</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>卷裝</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>綠色膠帶+高密度膜</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>裝潢養生/牆面門窗遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>防塵膠帶 2100mm</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>2100 mm × 25 y (22.8m)</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>卷裝</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>綠色膠帶+高密度膜</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>門窗/大型家具大面積遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>防塵膠帶 2700mm</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>2700 mm × 25 y (22.8m)</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>卷裝</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>綠色膠帶+高密度膜</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>工地工程/超大面積遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>其他類</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>防塵膠帶 3200mm</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>3200 mm × 25 y (22.8m)</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>卷裝</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>綠色膠帶+高密度膜</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>工程施工/最大面積養生遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
           <t>006</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>Scale Sheet</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Scale Sheet</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>專案洽詢</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>專案對接</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>專案客製</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>如有需求請聯繫專員專人對接</t>
         </is>

</xml_diff>